<commit_message>
Fixed continual learning and saved cap from paz_cap for each script
- continual learning fixed
- added paz_cap cap reference for each script
- general cleaning
</commit_message>
<xml_diff>
--- a/Simulazioni_RL/Strategy/paz_cap.xlsx
+++ b/Simulazioni_RL/Strategy/paz_cap.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,24 +469,36 @@
           <t>ppo conf</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>check_learning</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ripetizione</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>adult#001</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.09</v>
+          <t>adult#002</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>008/014</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>2048</v>
+        <v>1024</v>
       </c>
       <c r="D2" t="n">
-        <v>2048</v>
+        <v>1024</v>
       </c>
       <c r="E2" t="n">
-        <v>240822</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -502,6 +514,14 @@
         <is>
           <t>double</t>
         </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deleted redundant caps from checking_learning script
- Deleted redundant caps from checking_learning script
</commit_message>
<xml_diff>
--- a/Simulazioni_RL/Strategy/paz_cap.xlsx
+++ b/Simulazioni_RL/Strategy/paz_cap.xlsx
@@ -466,39 +466,37 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>ripetizione</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>ppo conf</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>check_learning</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>ripetizione</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>adult#002</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>008/014</t>
-        </is>
+          <t>adult#001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.09</v>
       </c>
       <c r="C2" t="n">
-        <v>1024</v>
+        <v>10240</v>
       </c>
       <c r="D2" t="n">
-        <v>1024</v>
+        <v>10240</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>11709</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -510,18 +508,18 @@
           <t>new</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>double</t>
-        </is>
+      <c r="H2" t="n">
+        <v>1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added random policy check
- added random policy check
</commit_message>
<xml_diff>
--- a/Simulazioni_RL/Strategy/paz_cap.xlsx
+++ b/Simulazioni_RL/Strategy/paz_cap.xlsx
@@ -466,37 +466,37 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>ppo conf</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>check_learning</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>ripetizione</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>ppo conf</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>check_learning</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>adult#001</t>
+          <t>adult#010</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.09</v>
+        <v>0.14</v>
       </c>
       <c r="C2" t="n">
-        <v>10240</v>
+        <v>1024</v>
       </c>
       <c r="D2" t="n">
-        <v>10240</v>
+        <v>1024</v>
       </c>
       <c r="E2" t="n">
-        <v>11709</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -508,18 +508,18 @@
           <t>new</t>
         </is>
       </c>
-      <c r="H2" t="n">
-        <v>1</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>single</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>